<commit_message>
Minor rev.1 pcb changes. Firmware progress
</commit_message>
<xml_diff>
--- a/Circuit Boards/BOM.xlsx
+++ b/Circuit Boards/BOM.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C1BE918-347B-4C70-BF9D-B1789E3B09FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="218" yWindow="900" windowWidth="21164" windowHeight="11662" xr2:uid="{8C143804-AE48-4691-8BB0-48B634FFE371}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{8C143804-AE48-4691-8BB0-48B634FFE371}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -802,28 +802,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">

</xml_diff>